<commit_message>
Doc: mise à jour du JDT
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_EmmaBlanchoud.xlsx
+++ b/Journal-de-Travail_EmmaBlanchoud.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pt70wvh\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pt70wvh\Documents\GitHub\Plot-those-lines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3311F96-CF80-46D3-9D1C-D59EE3938258}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F53311A8-FE85-4A46-BEA4-B0E5949E06BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="43">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -137,6 +137,39 @@
   </si>
   <si>
     <t>Blanchoud Emma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compréhension du projet et création de la maquette </t>
+  </si>
+  <si>
+    <t>Terminer la maquette et faire valider</t>
+  </si>
+  <si>
+    <t>Création du projet et essaie d'afficher un graphique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recherche sur blazor et recherche d'une librairie de graphique </t>
+  </si>
+  <si>
+    <t>Continuer dessayer d'afficher un graphique</t>
+  </si>
+  <si>
+    <t>Tester les extensions avec tout les types de projet pour essayer d'afficher un graphique</t>
+  </si>
+  <si>
+    <t>Création de l'application avec le modèle .NET MAUI Blazor Hybrid App et ajout d'un graphique de test</t>
+  </si>
+  <si>
+    <t>Aucune extension ne permet d'afficher un graphique (Blazorise, ChartJS)</t>
+  </si>
+  <si>
+    <t>Le problème ne vient pas des extensions mais du projet visual studio 2022</t>
+  </si>
+  <si>
+    <t>Modification des données du graphique</t>
+  </si>
+  <si>
+    <t>Recherche d'un autre moyen d'utiliser des graphiques avec Blazor</t>
   </si>
 </sst>
 </file>
@@ -1140,10 +1173,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>635</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2073,10 +2106,10 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0</c:v>
+                  <c:v>0.29444444444444445</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>0.7055555555555556</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4320,7 +4353,7 @@
       <c r="B3" s="86"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>0 heures 0 minutes</v>
+        <v>15 heures 0 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4335,15 +4368,15 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>0</v>
+        <v>720</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
@@ -4385,24 +4418,38 @@
       <c r="B7" s="26">
         <v>45903</v>
       </c>
-      <c r="C7" s="27"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="29"/>
-      <c r="F7" s="23"/>
+      <c r="C7" s="27">
+        <v>3</v>
+      </c>
+      <c r="D7" s="28">
+        <v>0</v>
+      </c>
+      <c r="E7" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="23" t="s">
+        <v>32</v>
+      </c>
       <c r="G7" s="38"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="62">
         <f>IF(ISBLANK(B8),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B8))</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" s="30">
-        <v>45903</v>
+        <v>45910</v>
       </c>
       <c r="C8" s="31"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="23"/>
+      <c r="D8" s="32">
+        <v>20</v>
+      </c>
+      <c r="E8" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="23" t="s">
+        <v>33</v>
+      </c>
       <c r="G8" s="39"/>
       <c r="M8" t="s">
         <v>15</v>
@@ -4417,15 +4464,23 @@
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="63">
         <f>IF(ISBLANK(B9),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B9))</f>
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="34">
-        <v>45903</v>
-      </c>
-      <c r="C9" s="35"/>
-      <c r="D9" s="36"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="23"/>
+        <v>45910</v>
+      </c>
+      <c r="C9" s="35">
+        <v>2</v>
+      </c>
+      <c r="D9" s="36">
+        <v>40</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>34</v>
+      </c>
       <c r="G9" s="40"/>
       <c r="M9" t="s">
         <v>16</v>
@@ -4440,15 +4495,21 @@
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="62">
         <f>IF(ISBLANK(B10),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B10))</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B10" s="30">
-        <v>45910</v>
+        <v>45917</v>
       </c>
       <c r="C10" s="31"/>
-      <c r="D10" s="32"/>
-      <c r="E10" s="33"/>
-      <c r="F10" s="23"/>
+      <c r="D10" s="32">
+        <v>45</v>
+      </c>
+      <c r="E10" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="F10" s="23" t="s">
+        <v>35</v>
+      </c>
       <c r="G10" s="39"/>
       <c r="M10" t="s">
         <v>17</v>
@@ -4463,16 +4524,26 @@
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="63">
         <f>IF(ISBLANK(B11),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B11))</f>
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B11" s="34">
-        <v>45910</v>
-      </c>
-      <c r="C11" s="35"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="37"/>
-      <c r="F11" s="23"/>
-      <c r="G11" s="40"/>
+        <v>45917</v>
+      </c>
+      <c r="C11" s="35">
+        <v>2</v>
+      </c>
+      <c r="D11" s="36">
+        <v>15</v>
+      </c>
+      <c r="E11" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="23" t="s">
+        <v>36</v>
+      </c>
+      <c r="G11" s="40" t="s">
+        <v>39</v>
+      </c>
       <c r="M11" t="s">
         <v>14</v>
       </c>
@@ -4486,16 +4557,26 @@
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="62">
         <f>IF(ISBLANK(B12),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B12))</f>
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="30">
-        <v>45917</v>
-      </c>
-      <c r="C12" s="31"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="39"/>
+        <v>45924</v>
+      </c>
+      <c r="C12" s="31">
+        <v>3</v>
+      </c>
+      <c r="D12" s="32">
+        <v>0</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F12" s="23" t="s">
+        <v>37</v>
+      </c>
+      <c r="G12" s="39" t="s">
+        <v>40</v>
+      </c>
       <c r="M12" t="s">
         <v>18</v>
       </c>
@@ -4509,15 +4590,21 @@
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="63">
         <f>IF(ISBLANK(B13),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B13))</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B13" s="34">
-        <v>45917</v>
+        <v>45931</v>
       </c>
       <c r="C13" s="35"/>
-      <c r="D13" s="36"/>
-      <c r="E13" s="37"/>
-      <c r="F13" s="23"/>
+      <c r="D13" s="36">
+        <v>20</v>
+      </c>
+      <c r="E13" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="23" t="s">
+        <v>42</v>
+      </c>
       <c r="G13" s="40"/>
       <c r="N13">
         <v>6</v>
@@ -4529,15 +4616,23 @@
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="62">
         <f>IF(ISBLANK(B14),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B14))</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B14" s="30">
-        <v>45924</v>
-      </c>
-      <c r="C14" s="31"/>
-      <c r="D14" s="32"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="23"/>
+        <v>45931</v>
+      </c>
+      <c r="C14" s="31">
+        <v>2</v>
+      </c>
+      <c r="D14" s="32">
+        <v>15</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="23" t="s">
+        <v>38</v>
+      </c>
       <c r="G14" s="39"/>
       <c r="N14">
         <v>7</v>
@@ -4549,15 +4644,21 @@
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="63">
         <f>IF(ISBLANK(B15),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B15))</f>
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B15" s="34">
-        <v>45924</v>
+        <v>45931</v>
       </c>
       <c r="C15" s="35"/>
-      <c r="D15" s="36"/>
-      <c r="E15" s="37"/>
-      <c r="F15" s="23"/>
+      <c r="D15" s="36">
+        <v>25</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="23" t="s">
+        <v>41</v>
+      </c>
       <c r="G15" s="40"/>
       <c r="N15">
         <v>8</v>
@@ -10916,15 +11017,15 @@
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="B6">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E6,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="C6">
         <f t="shared" ref="C6:C10" si="0">SUM(A6:B6)</f>
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="E6" s="70" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10932,11 +11033,11 @@
       </c>
       <c r="F6" s="71" t="str">
         <f>QUOTIENT(SUM(A6:B6),60)&amp;" h "&amp;TEXT(MOD(SUM(A6:B6),60), "00")&amp;" min"</f>
-        <v>0 h 00 min</v>
-      </c>
-      <c r="G6" s="72" t="e">
+        <v>4 h 25 min</v>
+      </c>
+      <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>#DIV/0!</v>
+        <v>0.29444444444444445</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -10953,15 +11054,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>0</v>
+        <v>540</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>635</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -10969,11 +11070,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>0 h 00 min</v>
-      </c>
-      <c r="G7" s="75" t="e">
+        <v>10 h 35 min</v>
+      </c>
+      <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>#DIV/0!</v>
+        <v>0.7055555555555556</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11008,9 +11109,9 @@
         <f t="shared" si="1"/>
         <v>0 h 00 min</v>
       </c>
-      <c r="G8" s="72" t="e">
+      <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11045,9 +11146,9 @@
         <f t="shared" si="1"/>
         <v>0 h 00 min</v>
       </c>
-      <c r="G9" s="75" t="e">
+      <c r="G9" s="75">
         <f t="shared" si="2"/>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="L9" s="55" t="str">
         <f>'Journal de travail'!M11</f>
@@ -11081,9 +11182,9 @@
         <f t="shared" ref="F10" si="4">QUOTIENT(SUM(A10:B10),60)&amp;" h "&amp;TEXT(MOD(SUM(A10:B10),60), "00")&amp;" min"</f>
         <v>0 h 00 min</v>
       </c>
-      <c r="G10" s="80" t="e">
+      <c r="G10" s="80">
         <f>SUM(A10:B10)/$C$11</f>
-        <v>#DIV/0!</v>
+        <v>0</v>
       </c>
       <c r="L10" s="69" t="s">
         <v>18</v>
@@ -11099,26 +11200,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>0</v>
+        <v>720</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>0</v>
+        <v>900</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>15 h 00 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0</v>
+        <v>0.17045454545454544</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11157,17 +11258,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005B1120F001D1794FAA6F4057E3355991" ma:contentTypeVersion="10" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="e4feb582a55ffdb09dc3e9683de3a0f4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f20a0681-8b2f-4a46-9dab-cf1520193f81" xmlns:ns3="932fafb7-d8e0-4a14-bee3-33aad5c71309" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7de6b5cf9a643ad34071d878fa0a2292" ns2:_="" ns3:_="">
     <xsd:import namespace="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
@@ -11356,6 +11446,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -11366,17 +11467,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA9A8432-080D-413D-841B-3BCFB73C0B04}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -11395,6 +11485,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
doc: mise à jour du journal de travail
</commit_message>
<xml_diff>
--- a/Journal-de-Travail_EmmaBlanchoud.xlsx
+++ b/Journal-de-Travail_EmmaBlanchoud.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pt70wvh\Documents\GitHub\Plot-those-lines\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EmmaB\Documents\GitHub\Plot-those-lines\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93356314-CD52-4C77-AC32-C493AD5BC173}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="705" windowWidth="29040" windowHeight="15840" xr2:uid="{6CC57B32-2488-5244-B7A6-FB7E808234AC}"/>
+    <workbookView xWindow="28680" yWindow="705" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Journal de travail" sheetId="1" r:id="rId1"/>
@@ -20,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Journal de travail'!$A$6:$G$6</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="53">
   <si>
     <t>Journal de travail</t>
   </si>
@@ -181,16 +180,34 @@
     <t>https://apexcharts.com/docs/options/</t>
   </si>
   <si>
-    <t>Ajouter un svg ou json dans le graphique (en cours)</t>
+    <t>Ajouter un csv ou json dans le graphique (en cours)</t>
+  </si>
+  <si>
+    <t>Ajout des csv et affichage des lignes dans le graphique</t>
+  </si>
+  <si>
+    <t>Ajout de l'option du choix des couleurs des lignes du graphique</t>
+  </si>
+  <si>
+    <t>Création d'un service pour gérer le filtre de date</t>
+  </si>
+  <si>
+    <t>Ajouter le composant du filtre</t>
+  </si>
+  <si>
+    <t>Modifier la home page pour utiliser le filtre</t>
+  </si>
+  <si>
+    <t>Test avec plusieurs fichiers avec différentes tranches de date</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="[$]dd/mm/yyyy;@" x16r2:formatCode16="[$-en-CH,1]dd/mm/yyyy;@"/>
-    <numFmt numFmtId="165" formatCode="[$]hh:mm;@" x16r2:formatCode16="[$-en-CH,1]hh:mm;@"/>
+    <numFmt numFmtId="164" formatCode="[$]dd/mm/yyyy;@"/>
+    <numFmt numFmtId="165" formatCode="[$]hh:mm;@"/>
     <numFmt numFmtId="166" formatCode="0\ &quot;h&quot;"/>
     <numFmt numFmtId="167" formatCode="dd\ mmm"/>
     <numFmt numFmtId="168" formatCode="00\ &quot;min&quot;"/>
@@ -642,6 +659,14 @@
     <xf numFmtId="10" fontId="11" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="16" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -652,20 +677,1020 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="0" xfId="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Lien hypertexte" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
+  <dxfs count="135">
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color theme="0"/>
@@ -764,7 +1789,6 @@
         <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -784,7 +1808,6 @@
         <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -803,7 +1826,6 @@
         <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <protection locked="0" hidden="0"/>
@@ -822,7 +1844,6 @@
         <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="168" formatCode="00\ &quot;min&quot;"/>
@@ -843,7 +1864,6 @@
         <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="166" formatCode="0\ &quot;h&quot;"/>
@@ -863,7 +1883,6 @@
         <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="167" formatCode="dd\ mmm"/>
@@ -883,7 +1902,6 @@
         <sz val="12"/>
         <color theme="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -918,13 +1936,96 @@
         <sz val="14"/>
         <color auto="1"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="2" tint="-9.9978637043366805E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCCCC00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="-0.24994659260841701"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="2" tint="-0.24994659260841701"/>
         </patternFill>
       </fill>
     </dxf>
@@ -956,7 +2057,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
@@ -1034,7 +2135,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000002-C1CD-1449-8ED0-F20983FC3F7F}"/>
               </c:ext>
@@ -1054,7 +2155,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-C1CD-1449-8ED0-F20983FC3F7F}"/>
               </c:ext>
@@ -1074,7 +2175,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000004-C1CD-1449-8ED0-F20983FC3F7F}"/>
               </c:ext>
@@ -1094,7 +2195,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000001-C1CD-1449-8ED0-F20983FC3F7F}"/>
               </c:ext>
@@ -1114,7 +2215,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000009-5CC6-E340-812C-86E0F7CCC2D7}"/>
               </c:ext>
@@ -1169,7 +2270,7 @@
                 <a:effectLst/>
               </c:spPr>
             </c:leaderLines>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
             </c:extLst>
           </c:dLbls>
@@ -1206,10 +2307,10 @@
                   <c:v>265</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>815</c:v>
+                  <c:v>1015</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1220,7 +2321,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-C1CD-1449-8ED0-F20983FC3F7F}"/>
             </c:ext>
@@ -1279,14 +2380,14 @@
     </c:legend>
     <c:plotVisOnly val="0"/>
     <c:dispBlanksAs val="gap"/>
-    <c:extLst>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1322,7 +2423,7 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
@@ -1401,7 +2502,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000001-4669-3541-AAAD-56FD9B888A4F}"/>
               </c:ext>
@@ -1423,7 +2524,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000003-4669-3541-AAAD-56FD9B888A4F}"/>
               </c:ext>
@@ -1445,7 +2546,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000005-4669-3541-AAAD-56FD9B888A4F}"/>
               </c:ext>
@@ -1467,7 +2568,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000007-4669-3541-AAAD-56FD9B888A4F}"/>
               </c:ext>
@@ -1487,7 +2588,7 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                 <c16:uniqueId val="{00000009-2877-BF46-A280-9AE4DAD1572E}"/>
               </c:ext>
@@ -1542,7 +2643,7 @@
                 <a:effectLst/>
               </c:spPr>
             </c:leaderLines>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
             </c:extLst>
           </c:dLbls>
@@ -1593,7 +2694,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000008-4669-3541-AAAD-56FD9B888A4F}"/>
             </c:ext>
@@ -1652,14 +2753,14 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:extLst>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1695,7 +2796,7 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <c:date1904 val="0"/>
   <c:lang val="fr-FR"/>
   <c:roundedCorners val="0"/>
@@ -1825,11 +2926,11 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000005-DDD9-EE41-8CD3-55D873EA4BB9}"/>
                 </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1846,11 +2947,11 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000004-DDD9-EE41-8CD3-55D873EA4BB9}"/>
                 </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1867,11 +2968,11 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000003-DDD9-EE41-8CD3-55D873EA4BB9}"/>
                 </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1888,11 +2989,11 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000002-DDD9-EE41-8CD3-55D873EA4BB9}"/>
                 </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -1909,11 +3010,11 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000000-3FA4-1D44-BA94-80D9B5CA27D4}"/>
                 </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
               </c:extLst>
             </c:dLbl>
             <c:numFmt formatCode="0%" sourceLinked="0"/>
@@ -1953,7 +3054,7 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="0"/>
               </c:ext>
@@ -2006,7 +3107,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-DDD9-EE41-8CD3-55D873EA4BB9}"/>
             </c:ext>
@@ -2058,11 +3159,11 @@
               <c:showSerName val="0"/>
               <c:showPercent val="0"/>
               <c:showBubbleSize val="0"/>
-              <c:extLst>
-                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+              <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
                 <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
                   <c16:uniqueId val="{00000001-3FA4-1D44-BA94-80D9B5CA27D4}"/>
                 </c:ext>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
               </c:extLst>
             </c:dLbl>
             <c:numFmt formatCode="00%" sourceLinked="0"/>
@@ -2100,7 +3201,7 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst>
+            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
                 <c15:showLeaderLines val="0"/>
               </c:ext>
@@ -2136,13 +3237,13 @@
                 <c:formatCode>0.00%</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>0.24537037037037038</c:v>
+                  <c:v>0.20384615384615384</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.75462962962962965</c:v>
+                  <c:v>0.78076923076923077</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>1.5384615384615385E-2</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -2153,7 +3254,7 @@
               </c:numCache>
             </c:numRef>
           </c:val>
-          <c:extLst>
+          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-DDD9-EE41-8CD3-55D873EA4BB9}"/>
             </c:ext>
@@ -2169,11 +3270,11 @@
         </c:dLbls>
         <c:gapWidth val="112"/>
         <c:overlap val="45"/>
-        <c:axId val="1745049904"/>
-        <c:axId val="686342815"/>
+        <c:axId val="175334664"/>
+        <c:axId val="175335056"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1745049904"/>
+        <c:axId val="175334664"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2216,7 +3317,7 @@
             <a:endParaRPr lang="fr-FR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="686342815"/>
+        <c:crossAx val="175335056"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2224,7 +3325,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="686342815"/>
+        <c:axId val="175335056"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2248,7 +3349,7 @@
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="1745049904"/>
+        <c:crossAx val="175334664"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2303,14 +3404,14 @@
     </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:extLst>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
           <c16r3:dispNaAsBlank val="1"/>
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4026,7 +5127,7 @@
         <xdr:cNvPr id="7" name="Chart 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6C2C91C8-8CC1-B699-56E8-6CF7F1B0F340}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{6C2C91C8-8CC1-B699-56E8-6CF7F1B0F340}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4062,7 +5163,7 @@
         <xdr:cNvPr id="8" name="Chart 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9ECD8AE3-367E-7D45-9847-71091F2762BE}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{9ECD8AE3-367E-7D45-9847-71091F2762BE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4105,7 +5206,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{685630F2-A1A1-EACE-5178-A329DD0FDCA2}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{685630F2-A1A1-EACE-5178-A329DD0FDCA2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4127,18 +5228,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}" name="Table1" displayName="Table1" ref="A6:G532" totalsRowShown="0" headerRowDxfId="17" tableBorderDxfId="16">
-  <autoFilter ref="A6:G532" xr:uid="{F2213DF1-F6B1-174C-AC17-4E96BE96C00D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A6:G532" totalsRowShown="0" headerRowDxfId="125" tableBorderDxfId="124">
+  <autoFilter ref="A6:G532"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{315BA4B4-9BD9-AB4E-8D40-FABFA0BB2AEA}" name="Semaine" dataDxfId="15">
+    <tableColumn id="1" name="Semaine" dataDxfId="123">
       <calculatedColumnFormula>IF(ISBLANK(B7),"",_xlfn.ISOWEEKNUM('Journal de travail'!$B7))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{503C31E9-854D-BF42-85AC-8DFA1376C4D8}" name="Jour" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{B35A0B98-71A0-BA4F-BFAB-00A05EA1F23A}" name="h.      " dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{BE4D837D-FC99-BA48-A82F-B8C8E4CE5BF8}" name="min." dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{A2DCC539-6D2A-B04A-BF8E-6FACE6268D1F}" name="Type" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{4EA406B9-7EF7-D547-AF98-5AD11BE168E9}" name="Description" dataDxfId="10"/>
-    <tableColumn id="7" xr3:uid="{1735360B-2647-6D42-A0E3-3425EE302FFD}" name="Remarques/problèmes" dataDxfId="9"/>
+    <tableColumn id="2" name="Jour" dataDxfId="122"/>
+    <tableColumn id="3" name="h.      " dataDxfId="121"/>
+    <tableColumn id="4" name="min." dataDxfId="120"/>
+    <tableColumn id="5" name="Type" dataDxfId="119"/>
+    <tableColumn id="6" name="Description" dataDxfId="118"/>
+    <tableColumn id="7" name="Remarques/problèmes" dataDxfId="117"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4328,7 +5429,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF2E8F1-C793-7E43-B3DE-C075053A97DA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:O532"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
@@ -4360,15 +5461,15 @@
       <c r="G1" s="11"/>
     </row>
     <row r="2" spans="1:15" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="88" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="86"/>
-      <c r="C2" s="84" t="s">
+      <c r="B2" s="88"/>
+      <c r="C2" s="86" t="s">
         <v>31</v>
       </c>
-      <c r="D2" s="84"/>
-      <c r="E2" s="84"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
       <c r="F2" s="5" t="s">
         <v>2</v>
       </c>
@@ -4377,13 +5478,13 @@
       </c>
     </row>
     <row r="3" spans="1:15" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A3" s="86" t="s">
+      <c r="A3" s="88" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="86"/>
+      <c r="B3" s="88"/>
       <c r="C3" s="67" t="str">
         <f>QUOTIENT(E4,60)&amp;" heures "&amp;MOD(E4,60)&amp;" minutes"</f>
-        <v>18 heures 0 minutes</v>
+        <v>21 heures 40 minutes</v>
       </c>
       <c r="D3" s="17"/>
       <c r="E3" s="3"/>
@@ -4398,24 +5499,24 @@
       <c r="B4" s="5"/>
       <c r="C4" s="17">
         <f>SUBTOTAL(9,$C$7:$C$531)*60</f>
-        <v>840</v>
+        <v>960</v>
       </c>
       <c r="D4" s="17">
         <f>SUBTOTAL(9,$D$7:$D$531)</f>
-        <v>240</v>
+        <v>340</v>
       </c>
       <c r="E4" s="24">
         <f>SUM(C4:D4)</f>
-        <v>1080</v>
+        <v>1300</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="6"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C5" s="85" t="s">
+      <c r="C5" s="87" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="85"/>
+      <c r="D5" s="87"/>
     </row>
     <row r="6" spans="1:15" s="15" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
@@ -4689,7 +5790,7 @@
       <c r="F15" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="87" t="s">
+      <c r="G15" s="84" t="s">
         <v>44</v>
       </c>
       <c r="N15">
@@ -4717,7 +5818,7 @@
       <c r="F16" s="23" t="s">
         <v>40</v>
       </c>
-      <c r="G16" s="88" t="s">
+      <c r="G16" s="85" t="s">
         <v>45</v>
       </c>
       <c r="O16">
@@ -4755,10 +5856,18 @@
         <v/>
       </c>
       <c r="B18" s="30"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="23"/>
+      <c r="C18" s="31">
+        <v>1</v>
+      </c>
+      <c r="D18" s="32">
+        <v>0</v>
+      </c>
+      <c r="E18" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="23" t="s">
+        <v>47</v>
+      </c>
       <c r="G18" s="39"/>
       <c r="O18">
         <v>50</v>
@@ -4771,9 +5880,15 @@
       </c>
       <c r="B19" s="34"/>
       <c r="C19" s="35"/>
-      <c r="D19" s="36"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="23"/>
+      <c r="D19" s="36">
+        <v>20</v>
+      </c>
+      <c r="E19" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="G19" s="40"/>
       <c r="O19">
         <v>55</v>
@@ -4785,10 +5900,16 @@
         <v/>
       </c>
       <c r="B20" s="30"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="23"/>
+      <c r="C20" s="35"/>
+      <c r="D20" s="36">
+        <v>40</v>
+      </c>
+      <c r="E20" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F20" s="23" t="s">
+        <v>48</v>
+      </c>
       <c r="G20" s="39"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -4797,10 +5918,18 @@
         <v/>
       </c>
       <c r="B21" s="34"/>
-      <c r="C21" s="35"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="37"/>
-      <c r="F21" s="23"/>
+      <c r="C21" s="31">
+        <v>1</v>
+      </c>
+      <c r="D21" s="32">
+        <v>15</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="23" t="s">
+        <v>49</v>
+      </c>
       <c r="G21" s="40"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -4810,9 +5939,15 @@
       </c>
       <c r="B22" s="30"/>
       <c r="C22" s="31"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="33"/>
-      <c r="F22" s="23"/>
+      <c r="D22" s="36">
+        <v>10</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F22" s="23" t="s">
+        <v>50</v>
+      </c>
       <c r="G22" s="39"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -4822,9 +5957,15 @@
       </c>
       <c r="B23" s="34"/>
       <c r="C23" s="35"/>
-      <c r="D23" s="36"/>
-      <c r="E23" s="37"/>
-      <c r="F23" s="23"/>
+      <c r="D23" s="32">
+        <v>15</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F23" s="23" t="s">
+        <v>51</v>
+      </c>
       <c r="G23" s="40"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
@@ -10943,49 +12084,165 @@
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E532">
-    <cfRule type="expression" dxfId="8" priority="1">
+  <conditionalFormatting sqref="E7:E19 E24:E532">
+    <cfRule type="expression" dxfId="134" priority="37">
       <formula>$E7="Absent"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="7" priority="2">
+    <cfRule type="expression" dxfId="133" priority="38">
       <formula>$E7="Autre"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="3" stopIfTrue="1">
+    <cfRule type="expression" dxfId="132" priority="39" stopIfTrue="1">
       <formula>$E7="Design"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="4" stopIfTrue="1">
+    <cfRule type="expression" dxfId="131" priority="40" stopIfTrue="1">
       <formula>$E7="Présentation"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="5" stopIfTrue="1">
+    <cfRule type="expression" dxfId="130" priority="41" stopIfTrue="1">
       <formula>$E7="Meeting"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="6" stopIfTrue="1">
+    <cfRule type="expression" dxfId="129" priority="42" stopIfTrue="1">
       <formula>$E7="Documentation"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="7" stopIfTrue="1">
+    <cfRule type="expression" dxfId="128" priority="43" stopIfTrue="1">
       <formula>$E7="Test"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="8" stopIfTrue="1">
+    <cfRule type="expression" dxfId="127" priority="44" stopIfTrue="1">
       <formula>$E7="Analyse"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="10" stopIfTrue="1">
+    <cfRule type="expression" dxfId="126" priority="46" stopIfTrue="1">
       <formula>$E7="Implémentation"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E23">
+    <cfRule type="expression" dxfId="71" priority="28">
+      <formula>$E23="Absent"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="70" priority="29">
+      <formula>$E23="Autre"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="69" priority="30" stopIfTrue="1">
+      <formula>$E23="Design"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="68" priority="31" stopIfTrue="1">
+      <formula>$E23="Présentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="67" priority="32" stopIfTrue="1">
+      <formula>$E23="Meeting"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="66" priority="33" stopIfTrue="1">
+      <formula>$E23="Documentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="65" priority="34" stopIfTrue="1">
+      <formula>$E23="Test"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="64" priority="35" stopIfTrue="1">
+      <formula>$E23="Analyse"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="63" priority="36" stopIfTrue="1">
+      <formula>$E23="Implémentation"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E22">
+    <cfRule type="expression" dxfId="53" priority="19">
+      <formula>$E22="Absent"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="52" priority="20">
+      <formula>$E22="Autre"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="51" priority="21" stopIfTrue="1">
+      <formula>$E22="Design"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="50" priority="22" stopIfTrue="1">
+      <formula>$E22="Présentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="49" priority="23" stopIfTrue="1">
+      <formula>$E22="Meeting"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="48" priority="24" stopIfTrue="1">
+      <formula>$E22="Documentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="47" priority="25" stopIfTrue="1">
+      <formula>$E22="Test"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="46" priority="26" stopIfTrue="1">
+      <formula>$E22="Analyse"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="27" stopIfTrue="1">
+      <formula>$E22="Implémentation"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E21">
+    <cfRule type="expression" dxfId="35" priority="10">
+      <formula>$E21="Absent"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="34" priority="11">
+      <formula>$E21="Autre"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="33" priority="12" stopIfTrue="1">
+      <formula>$E21="Design"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="32" priority="13" stopIfTrue="1">
+      <formula>$E21="Présentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="31" priority="14" stopIfTrue="1">
+      <formula>$E21="Meeting"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="30" priority="15" stopIfTrue="1">
+      <formula>$E21="Documentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="29" priority="16" stopIfTrue="1">
+      <formula>$E21="Test"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="28" priority="17" stopIfTrue="1">
+      <formula>$E21="Analyse"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="27" priority="18" stopIfTrue="1">
+      <formula>$E21="Implémentation"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E20">
+    <cfRule type="expression" dxfId="17" priority="1">
+      <formula>$E20="Absent"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="2">
+      <formula>$E20="Autre"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="3" stopIfTrue="1">
+      <formula>$E20="Design"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="4" stopIfTrue="1">
+      <formula>$E20="Présentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="5" stopIfTrue="1">
+      <formula>$E20="Meeting"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="6" stopIfTrue="1">
+      <formula>$E20="Documentation"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="7" stopIfTrue="1">
+      <formula>$E20="Test"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="8" stopIfTrue="1">
+      <formula>$E20="Analyse"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="9" priority="9" stopIfTrue="1">
+      <formula>$E20="Implémentation"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C532" xr:uid="{9D52E29F-610D-40B2-B3CC-F94A741DD978}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C7:C532">
       <formula1>$N$7:$N$15</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D532" xr:uid="{46510F84-8BCC-4BD6-9A19-9F03ACD74D05}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D7:D532">
       <formula1>$O$7:$O$19</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E532" xr:uid="{EBCA439E-C5F1-BC4C-88EE-2BB045537E3E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E7:E532">
       <formula1>$M$7:$M$12</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="G15" r:id="rId1" xr:uid="{866ECF82-C99A-4B22-A2A1-C777386B2AB3}"/>
-    <hyperlink ref="G16" r:id="rId2" xr:uid="{8672D784-C328-4A1C-B366-61295ADF3CA2}"/>
+    <hyperlink ref="G15" r:id="rId1"/>
+    <hyperlink ref="G16" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
@@ -10996,7 +12253,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D21D7432-C939-0D45-BAC2-A6A2196EA9C6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A2:N13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="18.75" x14ac:dyDescent="0.3"/>
@@ -11093,7 +12350,7 @@
       </c>
       <c r="G6" s="72">
         <f>SUM(A6:B6)/$C$11</f>
-        <v>0.24537037037037038</v>
+        <v>0.20384615384615384</v>
       </c>
       <c r="L6" s="51" t="str">
         <f>'Journal de travail'!M8</f>
@@ -11110,15 +12367,15 @@
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$C$7:$C$532)*60</f>
-        <v>660</v>
+        <v>780</v>
       </c>
       <c r="B7">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E7,'Journal de travail'!$D$7:$D$532)</f>
-        <v>155</v>
+        <v>235</v>
       </c>
       <c r="C7">
         <f t="shared" si="0"/>
-        <v>815</v>
+        <v>1015</v>
       </c>
       <c r="E7" s="73" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11126,11 +12383,11 @@
       </c>
       <c r="F7" s="74" t="str">
         <f t="shared" ref="F7:F11" si="1">QUOTIENT(SUM(A7:B7),60)&amp;" h "&amp;TEXT(MOD(SUM(A7:B7),60), "00")&amp;" min"</f>
-        <v>13 h 35 min</v>
+        <v>16 h 55 min</v>
       </c>
       <c r="G7" s="75">
         <f t="shared" ref="G7:G9" si="2">SUM(A7:B7)/$C$11</f>
-        <v>0.75462962962962965</v>
+        <v>0.78076923076923077</v>
       </c>
       <c r="L7" s="53" t="str">
         <f>'Journal de travail'!M9</f>
@@ -11151,11 +12408,11 @@
       </c>
       <c r="B8">
         <f>SUMIF('Journal de travail'!$E$7:$E$532,Plannification!E8,'Journal de travail'!$D$7:$D$532)</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="C8">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E8" s="76" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11163,11 +12420,11 @@
       </c>
       <c r="F8" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>0 h 00 min</v>
+        <v>0 h 20 min</v>
       </c>
       <c r="G8" s="72">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.5384615384615385E-2</v>
       </c>
       <c r="L8" s="54" t="str">
         <f>'Journal de travail'!M10</f>
@@ -11256,26 +12513,26 @@
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11">
         <f>SUM(A6:A10)</f>
-        <v>840</v>
+        <v>960</v>
       </c>
       <c r="B11">
         <f>SUM(B6:B10)</f>
-        <v>240</v>
+        <v>340</v>
       </c>
       <c r="C11">
         <f>SUM(A11:B11)</f>
-        <v>1080</v>
+        <v>1300</v>
       </c>
       <c r="E11" s="81" t="s">
         <v>29</v>
       </c>
       <c r="F11" s="71" t="str">
         <f t="shared" si="1"/>
-        <v>18 h 00 min</v>
+        <v>21 h 40 min</v>
       </c>
       <c r="G11" s="82">
         <f>C11/C12</f>
-        <v>0.20454545454545456</v>
+        <v>0.24621212121212122</v>
       </c>
       <c r="L11" s="56" t="s">
         <v>29</v>
@@ -11303,7 +12560,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67F31118-7D2C-C547-B9C9-EA2B04E048B8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -11314,14 +12571,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -11514,21 +12769,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f20a0681-8b2f-4a46-9dab-cf1520193f81">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="932fafb7-d8e0-4a14-bee3-33aad5c71309" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
-    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -11553,9 +12807,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{74326215-CB02-4E95-BFFB-9EC625B1BF0F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0453EC0E-0298-408B-815C-A1500DB4F5E9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="f20a0681-8b2f-4a46-9dab-cf1520193f81"/>
+    <ds:schemaRef ds:uri="932fafb7-d8e0-4a14-bee3-33aad5c71309"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>